<commit_message>
updated Power budgret and diagram
</commit_message>
<xml_diff>
--- a/docs/05-Power Budget/PowerBudgetSamBurns.xlsx
+++ b/docs/05-Power Budget/PowerBudgetSamBurns.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\umutb\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63169978-38F1-4046-943F-AA33919F9634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45F250FB-17EB-46AB-AB60-704830AAD3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="48">
   <si>
     <t>Team Number:</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Safety Margin</t>
   </si>
   <si>
-    <t>Total Current Required on +5V Rail</t>
-  </si>
-  <si>
     <t>c2. Regulator or Source Choice</t>
   </si>
   <si>
@@ -178,52 +175,37 @@
     <t xml:space="preserve">NHD-2.7-12864WDW3-MN </t>
   </si>
   <si>
-    <t>ESP32-S3-WOORM</t>
-  </si>
-  <si>
     <t xml:space="preserve"> +3.3V Power Rail</t>
   </si>
   <si>
     <t>3.3V regulator</t>
   </si>
   <si>
-    <t>AZ1117CH-3.3TRG1</t>
-  </si>
-  <si>
     <t>Total Remaining Current Available on +3.3V Rail</t>
   </si>
   <si>
     <t>Power Source 2 Selection</t>
   </si>
   <si>
-    <t>Power Source 3 Selection</t>
-  </si>
-  <si>
     <t>USB Port</t>
   </si>
   <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t>LP503030JU+PCM+2IC+NTC+MOL. 78172-3 50MM</t>
-  </si>
-  <si>
-    <t>3.7V</t>
-  </si>
-  <si>
     <t>Total Remaining Current Aailable on External Power Source 2</t>
   </si>
   <si>
     <t>Power Rails Connected to External Power Source 2</t>
   </si>
   <si>
-    <t>Power Rails Connected to External Power Source 3</t>
-  </si>
-  <si>
-    <t>Total Remaining Current Available on External Power Source 3</t>
-  </si>
-  <si>
     <t>C. Power Supply</t>
+  </si>
+  <si>
+    <t>ESP32-S3-WROOM</t>
+  </si>
+  <si>
+    <t>AP63203WU-7</t>
+  </si>
+  <si>
+    <t>Total Current Required on 3.3V Rail</t>
   </si>
 </sst>
 </file>
@@ -435,41 +417,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -496,16 +446,9 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -517,20 +460,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -895,25 +877,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A1" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="A1" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B2" s="44">
         <v>308</v>
       </c>
-      <c r="C2" s="16"/>
+      <c r="C2" s="45"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
@@ -921,10 +903,10 @@
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="13"/>
+      <c r="B3" s="42" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="43"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="3"/>
@@ -935,11 +917,11 @@
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="12"/>
-      <c r="D4" s="7"/>
+      <c r="B4" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="41"/>
+      <c r="D4" s="5"/>
       <c r="E4" s="1"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -949,10 +931,10 @@
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="38">
         <v>1</v>
       </c>
-      <c r="C5" s="10"/>
+      <c r="C5" s="39"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="3"/>
@@ -970,723 +952,679 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="11">
+        <v>1</v>
+      </c>
+      <c r="F9" s="10">
+        <v>800</v>
+      </c>
+      <c r="G9" s="10">
+        <f t="shared" ref="G9:G11" si="0">E9*F9</f>
+        <v>800</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="10"/>
+      <c r="B10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="23">
+      <c r="C10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="13">
         <v>1</v>
       </c>
-      <c r="F9" s="22">
-        <v>500</v>
-      </c>
-      <c r="G9" s="22">
-        <f t="shared" ref="G9:G11" si="0">E9*F9</f>
-        <v>500</v>
-      </c>
-      <c r="H9" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="22"/>
-      <c r="B10" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="25">
-        <v>1</v>
-      </c>
-      <c r="F10" s="24">
-        <v>15</v>
-      </c>
-      <c r="G10" s="22">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="H10" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="22"/>
-      <c r="B11" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="23">
-        <v>2</v>
-      </c>
-      <c r="F11" s="22">
-        <v>50</v>
-      </c>
-      <c r="G11" s="22">
+      <c r="F10" s="12">
+        <v>100</v>
+      </c>
+      <c r="G10" s="10">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H10" s="12" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="11">
+        <v>2</v>
+      </c>
+      <c r="F11" s="10">
+        <v>1</v>
+      </c>
+      <c r="G11" s="10">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="22"/>
-      <c r="B12" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" s="23"/>
-      <c r="F12" s="22">
-        <v>1350</v>
-      </c>
-      <c r="G12" s="22">
-        <v>1350</v>
-      </c>
-      <c r="H12" s="24" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="11"/>
+      <c r="F12" s="10">
+        <v>2000</v>
+      </c>
+      <c r="G12" s="10">
+        <v>2000</v>
+      </c>
+      <c r="H12" s="12" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="26"/>
-      <c r="B13" s="27"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
     </row>
     <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="21" t="s">
+      <c r="A15" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="F15" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="G15" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="17"/>
-      <c r="B16" s="22" t="s">
+      <c r="A16" s="7"/>
+      <c r="B16" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="11">
+        <v>1</v>
+      </c>
+      <c r="F16" s="10">
+        <v>800</v>
+      </c>
+      <c r="G16" s="10">
+        <f t="shared" ref="G16:G18" si="1">E16*F16</f>
+        <v>800</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7"/>
+      <c r="B17" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="23">
+      <c r="C17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="13">
         <v>1</v>
       </c>
-      <c r="F16" s="22">
-        <v>500</v>
-      </c>
-      <c r="G16" s="22">
-        <f t="shared" ref="G16:G18" si="1">E16*F16</f>
-        <v>500</v>
-      </c>
-      <c r="H16" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="17"/>
-      <c r="B17" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="25">
-        <v>1</v>
-      </c>
-      <c r="F17" s="24">
-        <v>15</v>
-      </c>
-      <c r="G17" s="22">
-        <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="H17" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="23">
-        <v>2</v>
-      </c>
-      <c r="F18" s="22">
-        <v>50</v>
-      </c>
-      <c r="G18" s="22">
+      <c r="F17" s="12">
+        <v>100</v>
+      </c>
+      <c r="G17" s="10">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="H18" s="24" t="s">
+      <c r="H17" s="12" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="11">
+        <v>2</v>
+      </c>
+      <c r="F18" s="10">
+        <v>1</v>
+      </c>
+      <c r="G18" s="10">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="22"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="24"/>
+      <c r="A19" s="10"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="22"/>
-      <c r="B20" s="32" t="s">
+      <c r="A20" s="10"/>
+      <c r="B20" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="22">
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="10">
         <f>SUM(G16:G19)</f>
-        <v>615</v>
-      </c>
-      <c r="H20" s="24" t="s">
+        <v>902</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="22"/>
-      <c r="B21" s="32" t="s">
+      <c r="A21" s="10"/>
+      <c r="B21" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="33"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="34">
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="20">
         <v>0.25</v>
       </c>
-      <c r="H21" s="34"/>
+      <c r="H21" s="20"/>
     </row>
     <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="35"/>
-      <c r="B22" s="36" t="s">
+      <c r="A22" s="21"/>
+      <c r="B22" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="10">
+        <f>G20*(1+G21)</f>
+        <v>1127.5</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="22"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="10"/>
+    </row>
+    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="22">
-        <f>G20*(1+G21)</f>
-        <v>768.75</v>
-      </c>
-      <c r="H22" s="24" t="s">
+      <c r="B24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="11"/>
+      <c r="F24" s="10">
+        <v>2000</v>
+      </c>
+      <c r="G24" s="10">
+        <v>2000</v>
+      </c>
+      <c r="H24" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="37"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="22"/>
-    </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="37" t="s">
+    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="22"/>
+      <c r="B25" s="33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="25">
+        <f>G24-G22</f>
+        <v>872.5</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="37"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="37"/>
+      <c r="E26" s="37"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="37"/>
+    </row>
+    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="10"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+    </row>
+    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="36"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+    </row>
+    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B29" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="24">
+        <v>3000</v>
+      </c>
+      <c r="G30" s="24">
+        <v>3000</v>
+      </c>
+      <c r="H30" s="23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="B31" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E24" s="23"/>
-      <c r="F24" s="22">
-        <v>1350</v>
-      </c>
-      <c r="G24" s="22">
-        <v>1350</v>
-      </c>
-      <c r="H24" s="24" t="s">
+      <c r="C31" s="13"/>
+      <c r="D31" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="F31" s="24">
+        <v>2000</v>
+      </c>
+      <c r="G31" s="24">
+        <v>2000</v>
+      </c>
+      <c r="H31" s="23"/>
+    </row>
+    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="27"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="32"/>
+      <c r="B34" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" s="11"/>
+      <c r="F34" s="10">
+        <v>2000</v>
+      </c>
+      <c r="G34" s="10">
+        <v>2000</v>
+      </c>
+      <c r="H34" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="37"/>
-      <c r="B25" s="41" t="s">
+    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="32"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="16"/>
+      <c r="B36" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="24">
+        <f>G30-SUM(G33:G35)</f>
+        <v>1000</v>
+      </c>
+      <c r="H36" s="23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="16"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+    </row>
+    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="23"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="32"/>
+      <c r="B39" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E39" s="11"/>
+      <c r="F39" s="10">
+        <v>2000</v>
+      </c>
+      <c r="G39" s="10">
+        <v>2000</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="32"/>
+      <c r="B40" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="40">
-        <f>G24-G22</f>
-        <v>581.25</v>
-      </c>
-      <c r="H25" s="24" t="s">
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="16"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="24">
+        <f>G31-SUM(G38:G40)</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="23" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="42"/>
-      <c r="B26" s="42"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="42"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="42"/>
-    </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="22"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-    </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-    </row>
-    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="E29" s="43" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="H29" s="20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="B30" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D30" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="E30" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="F30" s="39">
-        <v>3000</v>
-      </c>
-      <c r="G30" s="39">
-        <v>3000</v>
-      </c>
-      <c r="H30" s="38" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B31" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="E31" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="F31" s="39">
-        <v>2000</v>
-      </c>
-      <c r="G31" s="39">
-        <v>2000</v>
-      </c>
-      <c r="H31" s="38"/>
-    </row>
-    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="B32" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="C32" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="D32" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="E32" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="F32" s="39">
-        <v>450</v>
-      </c>
-      <c r="G32" s="40">
-        <v>1000</v>
-      </c>
-      <c r="H32" s="24"/>
-    </row>
-    <row r="33" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="45" t="s">
-        <v>23</v>
-      </c>
-      <c r="B33" s="38"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="24"/>
-    </row>
-    <row r="34" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="19"/>
-      <c r="B34" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E34" s="25">
-        <v>1</v>
-      </c>
-      <c r="F34" s="39">
-        <v>1350</v>
-      </c>
-      <c r="G34" s="40">
-        <f>E34*F34</f>
-        <v>1350</v>
-      </c>
-      <c r="H34" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="19"/>
-      <c r="B35" s="24"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="25"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="24"/>
-    </row>
-    <row r="36" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="28"/>
-      <c r="B36" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="39">
-        <f>G30-SUM(G33:G35)</f>
-        <v>1650</v>
-      </c>
-      <c r="H36" s="38" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="28"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="28"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="28"/>
-      <c r="H37" s="28"/>
-    </row>
-    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="45" t="s">
-        <v>50</v>
-      </c>
-      <c r="B38" s="38"/>
-      <c r="C38" s="38"/>
-      <c r="D38" s="25"/>
-      <c r="E38" s="25"/>
-      <c r="F38" s="39"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="24"/>
-    </row>
-    <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="19"/>
-      <c r="B39" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D39" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E39" s="25">
-        <v>1</v>
-      </c>
-      <c r="F39" s="39">
-        <v>1350</v>
-      </c>
-      <c r="G39" s="40">
-        <f>E39*F39</f>
-        <v>1350</v>
-      </c>
-      <c r="H39" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="19"/>
-      <c r="B40" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="C40" s="33"/>
-      <c r="D40" s="33"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="33"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="24"/>
-    </row>
-    <row r="41" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="28"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="39">
-        <f>G31-SUM(G38:G40)</f>
-        <v>650</v>
-      </c>
-      <c r="H41" s="38" t="s">
-        <v>13</v>
-      </c>
-    </row>
     <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="22"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
+      <c r="A42" s="10"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="45" t="s">
-        <v>51</v>
-      </c>
-      <c r="B43" s="38"/>
-      <c r="C43" s="38"/>
-      <c r="D43" s="25"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="40"/>
-      <c r="H43" s="24"/>
+      <c r="A43" s="31"/>
+      <c r="B43" s="23"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="25"/>
+      <c r="H43" s="12"/>
     </row>
     <row r="44" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="19"/>
-      <c r="B44" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D44" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E44" s="25">
-        <v>1</v>
-      </c>
-      <c r="F44" s="39">
-        <v>1350</v>
-      </c>
-      <c r="G44" s="40">
-        <f>E44*F44</f>
-        <v>1350</v>
-      </c>
-      <c r="H44" s="24" t="s">
-        <v>13</v>
-      </c>
+      <c r="A44" s="32"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="12"/>
     </row>
     <row r="45" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="19"/>
-      <c r="B45" s="24"/>
-      <c r="C45" s="22"/>
-      <c r="D45" s="25"/>
-      <c r="E45" s="23"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="24"/>
+      <c r="A45" s="32"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="12"/>
     </row>
     <row r="46" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="28"/>
-      <c r="B46" s="41" t="s">
-        <v>52</v>
-      </c>
-      <c r="C46" s="33"/>
-      <c r="D46" s="33"/>
-      <c r="E46" s="33"/>
-      <c r="F46" s="33"/>
-      <c r="G46" s="39">
-        <f>G32-SUM(G43:G45)</f>
-        <v>-350</v>
-      </c>
-      <c r="H46" s="38" t="s">
-        <v>13</v>
-      </c>
+      <c r="A46" s="16"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="24"/>
+      <c r="H46" s="23"/>
     </row>
     <row r="47" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="22"/>
-      <c r="B47" s="22"/>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="22"/>
+      <c r="A47" s="10"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
     </row>
     <row r="48" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1735,8 +1673,6 @@
     <row r="92" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="B40:F40"/>
     <mergeCell ref="A43:A45"/>
     <mergeCell ref="B46:F46"/>
     <mergeCell ref="A1:H1"/>
@@ -1754,6 +1690,8 @@
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B22:F22"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="B40:F40"/>
   </mergeCells>
   <conditionalFormatting sqref="G25">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>